<commit_message>
Adicionei qrcode em requiriment.txt
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3978A8F2-2990-4411-93EC-A8D6341BDB36}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9201A19C-C69B-4D47-85DD-E043A147E233}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="Etiqueta" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Etiqueta!$A$1:$B$25</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -775,6 +778,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -904,7 +910,7 @@
   <hyperlinks>
     <hyperlink ref="A25" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Foi começado a criar o identificador para que o QRcode consiga ler
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9201A19C-C69B-4D47-85DD-E043A147E233}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB158D59-C7DF-4E0B-9A76-F8B563A3BB40}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -435,57 +435,44 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>952499</xdr:colOff>
+      <xdr:colOff>546652</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>66262</xdr:rowOff>
+      <xdr:rowOff>33130</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1602270</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>182219</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="1789044" cy="679175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Imagem 6">
+        <xdr:cNvPr id="2" name="image1.png" title="Imagem">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AD8E9E6-6DDE-A848-4D40-BFB8C45A9F75}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC811D22-4B77-4415-A58C-1F3A21D62EB4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="15088" t="39298" r="17193" b="31579"/>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="952499" y="256762"/>
-          <a:ext cx="1598544" cy="687457"/>
+          <a:off x="546652" y="223630"/>
+          <a:ext cx="1789044" cy="679175"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
Mudança de ploanos, o usuário irá atualizar a planilha pela própria interface, estou mandano agora apenas a opção de input, nada mais
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luari\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA9081FE-15FC-47B7-ADE5-62948B2C70E0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,6 @@
     <sheet name="Etiqueta" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Etiqueta!$A$1:$B$25</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -134,7 +131,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,19 +170,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -329,10 +313,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -367,9 +352,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -401,7 +383,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>419573</xdr:colOff>
+      <xdr:colOff>5443</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -442,49 +424,58 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>546652</xdr:colOff>
+      <xdr:colOff>952499</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>33130</xdr:rowOff>
+      <xdr:rowOff>66262</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1789044" cy="679175"/>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1350065</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>182219</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="image1.png" title="Imagem">
+        <xdr:cNvPr id="7" name="Imagem 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC811D22-4B77-4415-A58C-1F3A21D62EB4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AD8E9E6-6DDE-A848-4D40-BFB8C45A9F75}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="15088" t="39298" r="17193" b="31579"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="546652" y="223630"/>
-          <a:ext cx="1789044" cy="679175"/>
+          <a:off x="952499" y="256762"/>
+          <a:ext cx="1598544" cy="687457"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -772,35 +763,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11"/>
-      <c r="B1" s="12"/>
+      <c r="A1" s="12"/>
+      <c r="B1" s="13"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="14"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="15"/>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="14"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="15"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="15"/>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="16"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="17"/>
     </row>
     <row r="6" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -827,72 +815,72 @@
       <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="11"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
     </row>
     <row r="23" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="6"/>
+      <c r="B23" s="7"/>
     </row>
     <row r="24" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="8"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="9"/>
     </row>
     <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="17"/>
+      <c r="B25" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -904,7 +892,7 @@
   <hyperlinks>
     <hyperlink ref="A25" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
   </hyperlinks>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
1º versão 100% finalizada do projeto funcional, agora falta adaptar para que a planilha da ODP represente ela mesma e não o operário,além de acrescentar as colunas chaves da aba historico na própria planilha modelo principal
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luari\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E375FC5-CF20-4743-862D-9BAD33F8C6CA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,22 +427,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>952499</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>66262</xdr:rowOff>
+      <xdr:colOff>430696</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>49696</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1350065</xdr:colOff>
+      <xdr:colOff>1749765</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>182219</xdr:rowOff>
+      <xdr:rowOff>259624</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Imagem 6">
+        <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AD8E9E6-6DDE-A848-4D40-BFB8C45A9F75}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C8850B1-533E-5426-0D6B-C018BB9E3325}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -450,23 +450,22 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="15088" t="39298" r="17193" b="31579"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="952499" y="256762"/>
-          <a:ext cx="1598544" cy="687457"/>
+          <a:off x="430696" y="49696"/>
+          <a:ext cx="2520047" cy="971928"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Modifiquei a etiqueta pra ficar mais estesticamente bonita
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E375FC5-CF20-4743-862D-9BAD33F8C6CA}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5576A705-831B-49C9-AC13-2AD3D137909E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,15 @@
     <sheet name="Etiqueta" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Etiqueta!$A$1:$B$31</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
   <si>
     <t>Data:</t>
   </si>
@@ -125,6 +128,9 @@
   </si>
   <si>
     <t>Máquina:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pesquisa de Qualidade: </t>
   </si>
 </sst>
 </file>
@@ -191,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -242,11 +248,65 @@
       </left>
       <right/>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -258,45 +318,10 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -307,17 +332,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -326,33 +357,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -382,8 +413,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>5443</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3108077</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -427,15 +458,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>430696</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>49696</xdr:rowOff>
+      <xdr:colOff>513523</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>41414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1749765</xdr:colOff>
+      <xdr:colOff>1904688</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>259624</xdr:rowOff>
+      <xdr:rowOff>300464</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -464,8 +495,208 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="430696" y="49696"/>
-          <a:ext cx="2520047" cy="971928"/>
+          <a:off x="513523" y="231914"/>
+          <a:ext cx="2153478" cy="830550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>19708</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>49696</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>715926</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>173934</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagem 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0DF434E-ADAE-C493-D53E-09A2C1108185}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19708" y="5810679"/>
+          <a:ext cx="696218" cy="695738"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1386941</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>57563</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1722529</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>12151</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Gráfico 12" descr="Contorno de rosto irritado com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9952094-FF4B-182B-D179-BED0B3C12EDD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId5"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2369748" y="6015018"/>
+          <a:ext cx="335588" cy="335588"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1914809</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>46292</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2259730</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>10213</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Gráfico 14" descr="Contorno de rosto nervoso com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34BD4FAE-DFFE-0C1F-A82B-D88B8ADCD25E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId7"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2897616" y="6003747"/>
+          <a:ext cx="344921" cy="344921"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2440280</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>47291</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2794043</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>20054</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Gráfico 16" descr="Contorno de rosto divertido com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D25D3F5-0AE5-392F-7210-70A6E823A351}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3423087" y="6004746"/>
+          <a:ext cx="353763" cy="353763"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -475,6 +706,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -762,137 +997,168 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B25"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12"/>
-      <c r="B1" s="13"/>
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
-      <c r="B4" s="15"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
-      <c r="B5" s="17"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="2"/>
     </row>
     <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="3"/>
+      <c r="B7" s="2"/>
     </row>
     <row r="8" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="3"/>
+      <c r="B8" s="2"/>
     </row>
     <row r="9" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12"/>
+      <c r="B10" s="13"/>
+    </row>
+    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12"/>
+      <c r="B11" s="13"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-    </row>
-    <row r="23" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+    </row>
+    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+    </row>
+    <row r="24" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+    </row>
+    <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="9"/>
-    </row>
-    <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="B25" s="9"/>
+    </row>
+    <row r="26" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+    </row>
+    <row r="27" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="5"/>
+      <c r="B27" s="7"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="17"/>
+      <c r="B28" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="18"/>
+      <c r="B29" s="15"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="18"/>
+      <c r="B30" s="15"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="19"/>
+      <c r="B31" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A23:B24"/>
-    <mergeCell ref="A10:B22"/>
-    <mergeCell ref="A1:B5"/>
+  <mergeCells count="6">
+    <mergeCell ref="A2:B5"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A25:B26"/>
+    <mergeCell ref="A10:B24"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A28:A31"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A25" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
+    <hyperlink ref="A27" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="260" scale="93" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>

</xml_diff>